<commit_message>
fullgame/FG-EMG-1: EMG1-E2E-01 阶段 1 出口旅程与出口模式清零
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/fg/#ChannelPort-通道端口.xlsx
+++ b/Configs/GameConfig/Datas/fg/#ChannelPort-通道端口.xlsx
@@ -2659,7 +2659,7 @@
         </is>
       </c>
       <c r="N38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39">
@@ -2717,7 +2717,7 @@
         </is>
       </c>
       <c r="N39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40">
@@ -3181,7 +3181,7 @@
         </is>
       </c>
       <c r="N47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="48">
@@ -3297,7 +3297,7 @@
         </is>
       </c>
       <c r="N49" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="50">
@@ -3355,7 +3355,7 @@
         </is>
       </c>
       <c r="N50" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="51">
@@ -3413,7 +3413,7 @@
         </is>
       </c>
       <c r="N51" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="52">
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="N52" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="53">
@@ -3529,7 +3529,7 @@
         </is>
       </c>
       <c r="N53" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="54">
@@ -4979,7 +4979,7 @@
         </is>
       </c>
       <c r="N78" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="79">
@@ -5037,7 +5037,7 @@
         </is>
       </c>
       <c r="N79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="80">
@@ -5269,7 +5269,7 @@
         </is>
       </c>
       <c r="N83" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="84">
@@ -5327,7 +5327,7 @@
         </is>
       </c>
       <c r="N84" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="85">

</xml_diff>